<commit_message>
Datos derivados: catalogo, registro, watchlist, comparador y brief
</commit_message>
<xml_diff>
--- a/data/pack/ca/amoniaco_ab.xlsx
+++ b/data/pack/ca/amoniaco_ab.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3569,6 +3569,61 @@
         </is>
       </c>
       <c r="K57" t="inlineStr">
+        <is>
+          <t>Contains information licensed under the Open Government Licence – Alberta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>amoniaco_ab</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Amoníaco anhidro con aplicador (Alberta)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1453.33</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>tonelada</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Alberta Agriculture and Irrigation — Weekly Market Review</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>OGL-Alberta</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
         <is>
           <t>Contains information licensed under the Open Government Licence – Alberta.</t>
         </is>
@@ -3672,7 +3727,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3738,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9">
@@ -3778,7 +3833,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>

</xml_diff>